<commit_message>
Expand equipment status effects
</commit_message>
<xml_diff>
--- a/JsonFile/Assets/ExcelFiles/AllItem_Master.xlsx
+++ b/JsonFile/Assets/ExcelFiles/AllItem_Master.xlsx
@@ -1309,7 +1309,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Option_003</t>
+          <t>화염 검</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>Test weapon: applies burn on hit</t>
+          <t>공격 적중 시 화상을 부여하는 테스트 무기</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -5517,7 +5517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="12.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5548,6 +5548,81 @@
           <t>Option_Type</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>StatusType</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ApplyMode</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>StackPolicy</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>MaxStack</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>TickInterval</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>TriggerType</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ValueMode</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>BaseChance</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ChancePerStack</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>BaseValue</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ValuePerStack</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ResistanceType</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>MaxRemoveCount</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="16.5" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -5570,6 +5645,55 @@
           <t>OnHit</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AddDamage</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -5592,6 +5716,60 @@
           <t>Passive</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>CriticalChance</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>CritChance</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" ht="16.5" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -5614,6 +5792,55 @@
           <t>OnHit</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Burn</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TimedTick</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>OnTick</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" ht="16.5" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -5636,6 +5863,55 @@
           <t>OnHit</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>HealOverTime</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>TimedTick</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>OnTick</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -5658,6 +5934,60 @@
           <t>Passive</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -5675,6 +6005,55 @@
           <t>Effect_006</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OneShotHPHeal</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>OnUse</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -5692,6 +6071,55 @@
           <t>Effect_007</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OneShotMPHeal</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>OnUse</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -5699,17 +6127,446 @@
           <t>Option_008</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>적중 시 대상의 다음 공격 1회 실패</t>
+        </is>
+      </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Effect_008</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ForcedMiss</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>OneShotState</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>99</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>BeforeAttack</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>StackCount</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1"/>
-    <row r="11" ht="16.5" customHeight="1"/>
-    <row r="12" ht="16.5" customHeight="1"/>
-    <row r="13" ht="16.5" customHeight="1"/>
-    <row r="14" ht="16.5" customHeight="1"/>
+    <row r="10" ht="16.5" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Option_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>출혈: 공격 시 스택 기반 확률로 최대 체력 비례 고정 피해</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Effect_009</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Bleed</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>99</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>OnAttack</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N10" t="n">
+        <v>7</v>
+      </c>
+      <c r="O10" t="n">
+        <v>2</v>
+      </c>
+      <c r="P10" t="n">
+        <v>2</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>BleedResist</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Option_010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>중독: 공격 시 스택 기반 확률로 최대 체력 비례 피해</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Effect_010</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Poison</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>99</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>OnAttack</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>100</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>PoisonResist</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="16.5" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Option_011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>신성: 공격 시 적 명중률 감소 및 자기 디버프 정화</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Effect_011</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Holy</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>99</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>OnAttack</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>7</v>
+      </c>
+      <c r="N12" t="n">
+        <v>2</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" ht="16.5" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Option_012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>재생: 공격 시 스택 기반 확률로 최대 체력 비례 회복</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Effect_012</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Regen</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>99</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>OnAttack</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>100</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="16.5" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Option_013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>빙결: 행동 전 확률로 행동 불가 및 속도 감소</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Effect_013</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Freeze</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>10</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>BeforeAttack</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>10</v>
+      </c>
+      <c r="N14" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>10</v>
+      </c>
+      <c r="P14" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>FreezeResist</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="15" ht="16.5" customHeight="1"/>
     <row r="16" ht="16.5" customHeight="1"/>
     <row r="17" ht="16.5" customHeight="1"/>

</xml_diff>

<commit_message>
Split option effect authoring data
</commit_message>
<xml_diff>
--- a/JsonFile/Assets/ExcelFiles/AllItem_Master.xlsx
+++ b/JsonFile/Assets/ExcelFiles/AllItem_Master.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Armor_Master" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item_Master" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Option_Master" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OptionEffect_Master" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -2364,21 +2365,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="11.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="16.5703125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="13.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="12.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="18.5703125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="17.42578125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="18.5703125" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="17.42578125" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="67.140625" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="11.7109375" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="12.7109375" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="8.7109375" customWidth="1" min="12" max="26"/>
+    <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="15" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="15" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="15" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="15" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="13" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="12" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="12" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="26"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="16.5" customHeight="1">
@@ -2923,7 +2938,53 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1"/>
+    <row r="12" ht="16.5" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Armor_011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>저항 테스트 갑옷</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>100</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Option_014</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>20</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Option_015</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>30</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>디버프 피해/출혈 저항 연결 테스트용 갑옷</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Armor</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>5</v>
+      </c>
+    </row>
     <row r="13" ht="16.5" customHeight="1"/>
     <row r="14" ht="16.5" customHeight="1"/>
     <row r="15" ht="16.5" customHeight="1"/>
@@ -5517,679 +5578,202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="12.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="34.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="19.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="14.28515625" customWidth="1" min="4" max="4"/>
+    <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="20" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="8.7109375" customWidth="1" min="5" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="16.5" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Option_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Option_Description</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Effect_ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Option_Type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>StatusType</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ApplyMode</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>StackPolicy</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>MaxStack</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Duration</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>TickInterval</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>TriggerType</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>ValueMode</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>BaseChance</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>ChancePerStack</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>BaseValue</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>ValuePerStack</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>StatType</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>ResistanceType</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>MaxRemoveCount</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="16.5" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Option_001</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>추가 공격력</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Effect_001</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>OnHit</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>AddDamage</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
+    </row>
+    <row r="3" ht="16.5" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Option_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>크리티컬 확률 증가</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Effect_002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16.5" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Option_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>공격 적중 시 최대 체력 비례 데미지 디버프</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Effect_003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>OnHit</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" ht="16.5" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Option_002</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>크리티컬 확률 증가</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Effect_002</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+    </row>
+    <row r="5" ht="16.5" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Option_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>최대 체력 비례 회복</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Effect_004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Option_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>공격 속도 증가</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Effect_005</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Passive</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>CriticalChance</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Passive</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Ignore</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>OnEquip</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>CritChance</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="16.5" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Option_003</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>공격 적중 시 최대 체력 비례 데미지 디버프</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Effect_003</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+    </row>
+    <row r="7" ht="16.5" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Option_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>체력을 회복합니다</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Effect_006</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Option_007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>정신력을 회복합니다</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Effect_007</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16.5" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Option_008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>적중 시 대상의 다음 공격 1회 실패</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Effect_008</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>OnHit</t>
         </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Burn</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>TimedTick</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Refresh</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>OnTick</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>PercentMaxHP</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="16.5" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Option_004</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>최대 체력 비례 회복</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Effect_004</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>OnHit</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>HealOverTime</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>TimedTick</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Refresh</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>5</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>OnTick</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>PercentMaxHP</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Option_005</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>공격 속도 증가</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Effect_005</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Passive</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>AttackSpeed</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Passive</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Ignore</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>OnEquip</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Percent</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Option_006</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>체력을 회복합니다</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Effect_006</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>OneShotHPHeal</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>OnUse</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Option_007</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>정신력을 회복합니다</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Effect_007</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>OneShotMPHeal</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>OnUse</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Flat</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Option_008</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>적중 시 대상의 다음 공격 1회 실패</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Effect_008</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>OnHit</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>ForcedMiss</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>OneShotState</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Stack</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>99</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>BeforeAttack</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>StackCount</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
@@ -6213,60 +5797,6 @@
           <t>OnHit</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Bleed</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Stacking</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Stack</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>99</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>OnAttack</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>PercentMaxHP</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N10" t="n">
-        <v>7</v>
-      </c>
-      <c r="O10" t="n">
-        <v>2</v>
-      </c>
-      <c r="P10" t="n">
-        <v>2</v>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>BleedResist</t>
-        </is>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -6289,60 +5819,6 @@
           <t>OnHit</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Poison</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Stacking</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Stack</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>99</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>OnAttack</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>PercentMaxHP</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
-        <v>100</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="n">
-        <v>1</v>
-      </c>
-      <c r="P11" t="n">
-        <v>1</v>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>PoisonResist</t>
-        </is>
-      </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -6365,55 +5841,6 @@
           <t>OnHit</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Holy</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Stacking</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Stack</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>99</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>OnAttack</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Percent</t>
-        </is>
-      </c>
-      <c r="M12" t="n">
-        <v>7</v>
-      </c>
-      <c r="N12" t="n">
-        <v>2</v>
-      </c>
-      <c r="O12" t="n">
-        <v>4</v>
-      </c>
-      <c r="P12" t="n">
-        <v>1</v>
-      </c>
-      <c r="S12" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -6436,55 +5863,6 @@
           <t>OnHit</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Regen</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Stacking</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Stack</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>99</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>OnAttack</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>PercentMaxHP</t>
-        </is>
-      </c>
-      <c r="M13" t="n">
-        <v>100</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="n">
-        <v>1</v>
-      </c>
-      <c r="P13" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -6507,70 +5885,95 @@
           <t>OnHit</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Freeze</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Stacking</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Stack</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>10</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>BeforeAttack</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Percent</t>
-        </is>
-      </c>
-      <c r="M14" t="n">
-        <v>10</v>
-      </c>
-      <c r="N14" t="n">
-        <v>5</v>
-      </c>
-      <c r="O14" t="n">
-        <v>10</v>
-      </c>
-      <c r="P14" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>Speed</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>FreezeResist</t>
-        </is>
-      </c>
-      <c r="S14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="16.5" customHeight="1"/>
-    <row r="16" ht="16.5" customHeight="1"/>
-    <row r="17" ht="16.5" customHeight="1"/>
-    <row r="18" ht="16.5" customHeight="1"/>
+    </row>
+    <row r="15" ht="16.5" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Option_014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>디버프 피해 저항</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Effect_014</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16.5" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Option_015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>출혈 저항</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Effect_014</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Option_016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>중독 저항</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Effect_014</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16.5" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Option_017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>빙결 저항</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Effect_014</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+    </row>
     <row r="19" ht="16.5" customHeight="1"/>
     <row r="20" ht="16.5" customHeight="1"/>
     <row r="21" ht="16.5" customHeight="1"/>
@@ -7557,4 +6960,1120 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Option_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>StatusType</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ApplyMode</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>StackPolicy</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>MaxStack</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>TickInterval</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>TriggerType</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ValueMode</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>BaseChance</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ChancePerStack</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>BaseValue</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ValuePerStack</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ResistanceType</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>MaxRemoveCount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Option_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AddDamage</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Option_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CriticalChance</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>CritChance</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Option_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Burn</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TimedTick</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>OnTick</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Option_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HealOverTime</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TimedTick</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>OnTick</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Option_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Option_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OneShotHPHeal</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>OnUse</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Option_007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>OneShotMPHeal</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>OnUse</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Option_008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ForcedMiss</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>OneShotState</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>99</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>BeforeAttack</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>StackCount</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Option_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bleed</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>99</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>OnAttack</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>BleedResist</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Option_010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Poison</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>99</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>OnAttack</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>100</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>PoisonResist</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Option_011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Holy</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>99</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>OnAttack</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>7</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>4</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Option_012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Regen</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>99</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>OnAttack</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>PercentMaxHP</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>100</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Option_013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Freeze</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Stacking</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Stack</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>10</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>BeforeAttack</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>10</v>
+      </c>
+      <c r="M14" t="n">
+        <v>5</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>FreezeResist</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Option_014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DebuffDamageResist</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>DebuffDamageResist</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Option_015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BleedResist</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>BleedResist</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Option_016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PoisonResist</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>PoisonResist</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Option_017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>FreezeResist</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Ignore</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>FreezeResist</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>